<commit_message>
Update audio and spreadsheet assets for HI02H04_L01_S01
</commit_message>
<xml_diff>
--- a/HTML_Self Review Checklist - HI02H04_L01_S01 (marked).xlsx
+++ b/HTML_Self Review Checklist - HI02H04_L01_S01 (marked).xlsx
@@ -1857,19 +1857,19 @@
 शाबाश! आज तो कमाल कर दिया!</t>
         </is>
       </c>
-      <c r="C60" s="17" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="C60" s="14" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="D60" s="13" t="inlineStr">
         <is>
-          <t>vo_well_done says “शाबाश! आपने चित्रों और वाक्यों को मिलाना सीख लिया!” — not one of the three standard lines.</t>
+          <t>Since 2026-10-09 the closing line is MTG2A04_L01_S01’s own vo_cel_prompt: “बहुत बढ़िया, दोस्त! तुमने कमाल कर दिया!” (2.94 s), applied under the vo_well_done id with that card’s lip-sync frames.</t>
         </is>
       </c>
       <c r="E60" s="13" t="inlineStr">
         <is>
-          <t>Re-record with one of the three (e.g. “शाबाश! आज तो कमाल कर दिया!”). Note: the other two use तुम forms, which conflicts with the आप ruling; prefer the third.</t>
+          <t>The line is −2.5 dB louder than this lesson’s other clips (−15.8 vs ≈−18 LUFS); level-match if the reviewer hears the jump.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add pulsating effect for the Next button and update checklist for consistency
</commit_message>
<xml_diff>
--- a/HTML_Self Review Checklist - HI02H04_L01_S01 (marked).xlsx
+++ b/HTML_Self Review Checklist - HI02H04_L01_S01 (marked).xlsx
@@ -1226,21 +1226,17 @@
           <t xml:space="preserve">The Next button pulsates immediately after the VO and the CTA for a screen is complete. </t>
         </is>
       </c>
-      <c r="C27" s="17" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="C27" s="14" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="D27" s="13" t="inlineStr">
         <is>
-          <t>No pulse on आगे when it becomes active; a hand taps it after 4.5 s of inactivity (nudgeNavBtn, line 1390).</t>
-        </is>
-      </c>
-      <c r="E27" s="13" t="inlineStr">
-        <is>
-          <t>Add a pulse class on setNavActive(true) (e.g. the sgBtnPulse keyframes on .nav-btn.active) and keep the hand as the 7 s idle nudge.</t>
-        </is>
-      </c>
+          <t>Since 2026-10-09 the enabled आगे pulses the moment it is enabled ([NAV-PULSE]: the sentence chip’s cue keyframes, scale 1 → 1.10, 0.8 s, on the enabled art layer); the hand nudge still follows after 4.5 s of inactivity.</t>
+        </is>
+      </c>
+      <c r="E27" s="13" t="inlineStr"/>
     </row>
     <row r="28" ht="15" customHeight="1">
       <c r="A28" s="13" t="inlineStr"/>

</xml_diff>